<commit_message>
updated template and added email send feature
</commit_message>
<xml_diff>
--- a/Invoice_template.xlsx
+++ b/Invoice_template.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="3640" yWindow="600" windowWidth="21960" windowHeight="13800" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="3620" yWindow="600" windowWidth="21980" windowHeight="13800" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Invoice" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Invoice" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="ColumnTitle1">InvoiceDetails[[#Headers],[Details]]</definedName>
@@ -132,7 +132,7 @@
       <alignment horizontal="left"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
@@ -152,31 +152,25 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="165" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="8">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="6">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="4">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="9">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="9">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="9">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="4">
-      <alignment horizontal="right" indent="1"/>
-    </xf>
-    <xf numFmtId="10" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="6">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="8">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="4">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="10">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -573,7 +567,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr codeName="Sheet1">
     <tabColor theme="4"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -582,47 +576,47 @@
   <dimension ref="B1:C21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="30" customHeight="1"/>
   <cols>
-    <col width="2.5" customWidth="1" style="17" min="1" max="1"/>
-    <col width="50.6640625" customWidth="1" style="17" min="2" max="2"/>
-    <col width="30.5" customWidth="1" style="17" min="3" max="3"/>
-    <col width="2.5" customWidth="1" style="17" min="4" max="4"/>
+    <col width="2.5" customWidth="1" style="13" min="1" max="1"/>
+    <col width="50.6640625" customWidth="1" style="13" min="2" max="2"/>
+    <col width="30.5" customWidth="1" style="13" min="3" max="3"/>
+    <col width="2.5" customWidth="1" style="13" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" s="17">
+    <row r="1" ht="30" customHeight="1" s="13">
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>INVOICE #3676</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="50.25" customHeight="1" s="17">
+          <t>INVOICE #3678</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="50.25" customHeight="1" s="13">
       <c r="B2" s="7" t="inlineStr">
         <is>
           <t>Funky's Electrical</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="30" customHeight="1" s="17">
+    <row r="3" ht="30" customHeight="1" s="13">
       <c r="B3" s="0" t="inlineStr">
         <is>
           <t>5924 Ashton Woods Cir., Milton, FL 32570</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="18" customHeight="1" s="17">
+    <row r="4" ht="18" customHeight="1" s="13">
       <c r="B4" s="6" t="inlineStr">
         <is>
           <t>(850) 207-1800</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="25" customHeight="1" s="17">
+    <row r="5" ht="25" customHeight="1" s="13">
       <c r="B5" s="3">
         <f>TODAY()</f>
         <v/>
       </c>
     </row>
-    <row r="6" ht="30" customHeight="1" s="17">
+    <row r="6" ht="30" customHeight="1" s="13">
       <c r="B6" s="5" t="inlineStr">
         <is>
           <t>BILL TO</t>
@@ -634,34 +628,30 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="18" customHeight="1" s="17">
+    <row r="7" ht="18" customHeight="1" s="13">
       <c r="B7" s="0" t="inlineStr">
         <is>
-          <t>Allan Raynor</t>
-        </is>
-      </c>
-      <c r="C7" s="18" t="inlineStr">
-        <is>
-          <t>sdfg</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="30" customHeight="1" s="17">
+          <t>Wayne Campbell</t>
+        </is>
+      </c>
+      <c r="C7" s="16" t="inlineStr">
+        <is>
+          <t>Generator Work</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1" s="13">
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t>1292 Point E Cir
-Gulf Breeze, Fl, 32563</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="18" customHeight="1" s="17">
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>785-565-8828</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="30" customHeight="1" s="17">
+          <t>7373 Chumuckla Hwy
+Pace, Fl, 32571</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1" s="13">
+      <c r="B9" s="6" t="n"/>
+    </row>
+    <row r="10" ht="30" customHeight="1" s="13">
       <c r="B10" s="0" t="inlineStr">
         <is>
           <t>Salesperson</t>
@@ -673,7 +663,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="30" customHeight="1" s="17">
+    <row r="11" ht="30" customHeight="1" s="13">
       <c r="B11" s="0" t="inlineStr">
         <is>
           <t>Gary Funkhouser</t>
@@ -685,7 +675,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="30" customHeight="1" s="17">
+    <row r="12" ht="30" customHeight="1" s="13">
       <c r="B12" s="2" t="inlineStr">
         <is>
           <t>Details</t>
@@ -697,102 +687,90 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="30" customHeight="1" s="17">
+    <row r="13" ht="30" customHeight="1" s="13">
       <c r="B13" s="0" t="inlineStr">
         <is>
-          <t>dsf</t>
-        </is>
-      </c>
-      <c r="C13" s="15" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="14" ht="30" customHeight="1" s="17">
-      <c r="B14" s="13" t="inlineStr">
+          <t>Generator Work</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="n">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1" s="13">
+      <c r="B14" s="4" t="inlineStr">
         <is>
           <t>SUBTOTAL</t>
         </is>
       </c>
-      <c r="C14" s="15">
+      <c r="C14" s="8">
         <f>SUBTOTAL(109,InvoiceDetails[AMOUNT])</f>
         <v/>
       </c>
     </row>
-    <row r="15" ht="30" customHeight="1" s="17">
-      <c r="B15" s="13" t="inlineStr">
+    <row r="15" ht="30" customHeight="1" s="13">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>SALES TAX</t>
         </is>
       </c>
-    </row>
-    <row r="16" ht="30" customHeight="1" s="17">
-      <c r="B16" s="13" t="inlineStr">
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1" s="13">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-    </row>
-    <row r="17" ht="30" customHeight="1" s="17">
-      <c r="B17" s="16" t="n"/>
-    </row>
-    <row r="18" ht="30" customHeight="1" s="17">
-      <c r="B18" s="10">
+      <c r="C16" s="8">
+        <f>SUM(C14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1" s="13">
+      <c r="B17" s="10" t="n"/>
+    </row>
+    <row r="18" ht="30" customHeight="1" s="13">
+      <c r="B18" s="12">
         <f>"Make all checks payable to "&amp; Company_Name</f>
         <v/>
       </c>
     </row>
-    <row r="19" ht="30" customHeight="1" s="17">
-      <c r="B19" s="11" t="inlineStr">
+    <row r="19" ht="30" customHeight="1" s="13">
+      <c r="B19" s="14" t="inlineStr">
         <is>
           <t>If you have any questions concerning this invoice, use the following contact information:</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="30" customHeight="1" s="17">
-      <c r="B20" s="12" t="inlineStr">
+    <row r="20" ht="30" customHeight="1" s="13">
+      <c r="B20" s="15" t="inlineStr">
         <is>
           <t>Gary Funkhouser, (850) 207-1800, funkyselectrical@gmail.com
 License # EC13005709</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="30" customHeight="1" s="17">
+    <row r="21" ht="30" customHeight="1" s="13">
       <c r="B21" s="2" t="inlineStr">
         <is>
           <t>THANK YOU FOR YOUR BUSINESS!</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="14" customHeight="1" s="17"/>
-    <row r="23" ht="14" customHeight="1" s="17"/>
-    <row r="24" ht="14" customHeight="1" s="17"/>
-    <row r="25" ht="14" customHeight="1" s="17"/>
-    <row r="26" ht="14" customHeight="1" s="17"/>
-    <row r="27" ht="14" customHeight="1" s="17"/>
-    <row r="28" ht="14" customHeight="1" s="17"/>
-    <row r="29" ht="14" customHeight="1" s="17"/>
-    <row r="30" ht="14" customHeight="1" s="17"/>
-    <row r="31" ht="14" customHeight="1" s="17"/>
-    <row r="32" ht="14" customHeight="1" s="17"/>
-    <row r="33" ht="14" customHeight="1" s="17"/>
-    <row r="34" ht="14" customHeight="1" s="17"/>
-    <row r="35" ht="14" customHeight="1" s="17"/>
-    <row r="36" ht="14" customHeight="1" s="17"/>
-    <row r="37" ht="14" customHeight="1" s="17"/>
-    <row r="38" ht="14" customHeight="1" s="17"/>
-    <row r="39" ht="14" customHeight="1" s="17"/>
-    <row r="40" ht="14" customHeight="1" s="17"/>
-    <row r="41" ht="14" customHeight="1" s="17"/>
-    <row r="42" ht="14" customHeight="1" s="17"/>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="B15:C15"/>
-    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B20:C20"/>
     <mergeCell ref="C7:C9"/>
-    <mergeCell ref="B17:C17"/>
   </mergeCells>
-  <dataValidations count="18">
-    <dataValidation sqref="A2:A1048576 B18:C1048576 C1:C5 D1:XFD8 D9:H9 D10:XFD1048576 J9:XFD9" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0"/>
+  <dataValidations count="24">
+    <dataValidation sqref="A2:A1048576 B21:C1048576 C1:C5 D1:XFD8 D9:H9 D10:XFD1048576 J9:XFD9" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0"/>
     <dataValidation sqref="A1" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" prompt="Create an Invoice in this worksheet. Enter invoice details, item descriptions, amount, tax rate, and any other cost. Subtotal and Total are automatically calculated"/>
     <dataValidation sqref="B1" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" prompt="Enter Invoice Number in this cell. Enter Invoice Company &amp; Customer details in cells below"/>
     <dataValidation sqref="B2" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" prompt="Enter Invoice Company Name in this cell"/>
@@ -803,9 +781,15 @@
     <dataValidation sqref="C6" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" prompt="Enter Invoice Product Description in cell below"/>
     <dataValidation sqref="C7:C10" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" prompt="Enter Product Description in this cell"/>
     <dataValidation sqref="B8" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" prompt="Enter Bill To Address, City, State, and Zip Code in this cell"/>
-    <dataValidation sqref="B15:C15" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" prompt="Company Name is automatically appended in this cell"/>
-    <dataValidation sqref="B16:C16" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" prompt="Enter Contact details in cell below"/>
-    <dataValidation sqref="B17:C17" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" prompt="Enter Contact Name, Phone Number, and Email in this cell"/>
+    <dataValidation sqref="B14" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" prompt="Subtotal is automatically calculated in cell at right"/>
+    <dataValidation sqref="C14" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" prompt="Subtotal is automatically calculated in this cell"/>
+    <dataValidation sqref="B15" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" prompt="Enter Tax Rate in cell at right"/>
+    <dataValidation sqref="C15" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" prompt="Enter Tax Rate in this cell"/>
+    <dataValidation sqref="B16" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" prompt="Total is automatically calculated in cell at right"/>
+    <dataValidation sqref="C16" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" prompt="Total is automatically calculated in this cell"/>
+    <dataValidation sqref="B18:C18" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" prompt="Company Name is automatically appended in this cell"/>
+    <dataValidation sqref="B19:C19" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" prompt="Enter Contact details in cell below"/>
+    <dataValidation sqref="B20:C20" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" prompt="Enter Contact Name, Phone Number, and Email in this cell"/>
     <dataValidation sqref="B9:B10" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" prompt="Enter Bill To Phone number in this cell"/>
     <dataValidation sqref="B7" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" prompt="Enter Bill To Customer Name or Company Name in this cell"/>
     <dataValidation sqref="C12:C13" showDropDown="0" showInputMessage="1" showErrorMessage="1" allowBlank="0" prompt="Enter Amount in this column under this heading for each description in column B. Enter Tax Rate &amp; any Other cost in cell below the table to calculate Subtotal and Total amount"/>
@@ -823,8 +807,8 @@
     <firstFooter/>
   </headerFooter>
   <tableParts count="2">
-    <tablePart r:id="rId1"/>
-    <tablePart r:id="rId2"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>